<commit_message>
Se sube requisitos No Funcionales y de seguridad
</commit_message>
<xml_diff>
--- a/01_PRIMER_PARCIAL/01_DOCUMENTACION/02_REQUISITOS/02_REQUISITOS_NO_FUNCIONALES_V01.xlsx
+++ b/01_PRIMER_PARCIAL/01_DOCUMENTACION/02_REQUISITOS/02_REQUISITOS_NO_FUNCIONALES_V01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josecito/Desktop/ESPE/SEPTIMO/SOFTWARE SEGURO/36902-DESARROLLO_SOFTWARE_SEGURO-PROYECTOS/01_PRIMER_PARCIAL/01_DOCUMENTACION/02_REQUISITOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2B5595-1D05-9D4F-86C2-166996CA4FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC7B2B2-419C-2241-8E5B-92F6AD9F95D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="16480" activeTab="1" xr2:uid="{401C71C4-BAB8-A749-A636-1C285FBB789A}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="16640" activeTab="1" xr2:uid="{401C71C4-BAB8-A749-A636-1C285FBB789A}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUISITOS FUNCIONALES" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="117">
   <si>
     <t>Código</t>
   </si>
@@ -196,18 +196,224 @@
   </si>
   <si>
     <t>El sistema deberá emitir alertas automáticas dirigidas al administrador y a los participantes pertinentes cuando se detecte un archivo anómalo o un evento de seguridad crítico.</t>
+  </si>
+  <si>
+    <t>Atributo</t>
+  </si>
+  <si>
+    <t>Requisito no funcional</t>
+  </si>
+  <si>
+    <t>Criterio de aceptación</t>
+  </si>
+  <si>
+    <t>RNF-01</t>
+  </si>
+  <si>
+    <t>Rendimiento (Mensajería)</t>
+  </si>
+  <si>
+    <t>El sistema deberá procesar, cifrar y entregar los mensajes de texto a través de WebSockets con una latencia imperceptible en tiempo real.</t>
+  </si>
+  <si>
+    <t>RNF-02</t>
+  </si>
+  <si>
+    <t>Rendimiento (Análisis multimedia)</t>
+  </si>
+  <si>
+    <t>El pipeline de análisis esteganográfico (entropía de Shannon y chi-cuadrado) y recodificación destructiva de imágenes debe ejecutarse sin bloquear el flujo de mensajería.</t>
+  </si>
+  <si>
+    <t>Tiempo medio de detección y procesado (MTTD) menor a 1.5 segundos para imágenes PNG/JPG de hasta 5 MB en el 90% de las solicitudes.</t>
+  </si>
+  <si>
+    <t>RNF-03</t>
+  </si>
+  <si>
+    <t>Disponibilidad</t>
+  </si>
+  <si>
+    <t>Los servicios de autenticación, control de salas y pasarela de mensajería en tiempo real deberán ofrecer alta disponibilidad operativa.</t>
+  </si>
+  <si>
+    <t>Disponibilidad mensual mínima de 99.5% de tiempo en línea (uptime), tolerando un tiempo de inactividad no planificado inferior a 3.6 horas/mes.</t>
+  </si>
+  <si>
+    <t>RNF-04</t>
+  </si>
+  <si>
+    <t>Escalabilidad</t>
+  </si>
+  <si>
+    <t>La arquitectura del sistema deberá soportar el incremento de salas y conexiones concurrentes mediante contenedores y gestión de sesiones distribuidas en memoria (Redis).</t>
+  </si>
+  <si>
+    <t>Capacidad para sostener al menos 500 conexiones WebSocket concurrentes en 50 salas simultáneas sin superar el 75% de CPU ni el 80% de RAM en el host de ejecución.</t>
+  </si>
+  <si>
+    <t>RNF-05</t>
+  </si>
+  <si>
+    <t>Recuperación ante fallos</t>
+  </si>
+  <si>
+    <t>El sistema deberá restablecer el servicio de mensajería y la coherencia del estado de las salas de forma desatendida ante caídas del gateway o contenedores de procesamiento.</t>
+  </si>
+  <si>
+    <t>Tiempo Objetivo de Recuperación (RTO) menor a 60 segundos tras fallo imprevisto mediante reinicio automático orquestado de Docker, preservando la integridad de datos persistidos.</t>
+  </si>
+  <si>
+    <t>RNF-06</t>
+  </si>
+  <si>
+    <t>Seguridad (Cifrado y canal)</t>
+  </si>
+  <si>
+    <t>Las comunicaciones en tránsito y el intercambio de llaves deben protegerse contra ataques Man-in-the-Middle y fugas de datos mediante suites criptográficas modernas.</t>
+  </si>
+  <si>
+    <t>Implementación exclusiva de TLS 1.3 con certificados válidos y cifrado autenticado simétrico AES-256-GCM / ChaCha20-Poly1305, sin suites obsoletas (calificación 'A' en SSL Labs / testssl).</t>
+  </si>
+  <si>
+    <t>RNF-07</t>
+  </si>
+  <si>
+    <t>Seguridad (Aislamiento / Sandbox)</t>
+  </si>
+  <si>
+    <t>El análisis de archivos multimedia no confiables y el proceso de sanitización destructiva deben aislarse para evitar escapes de contenedor (RSG-06, RSG-14).</t>
+  </si>
+  <si>
+    <t>Ejecución obligatoria en contenedores Docker efímeros sin privilegios (no-root), sistema de archivos en solo lectura (read-only rootfs) y perfiles restrictivos de Seccomp y AppArmor activos.</t>
+  </si>
+  <si>
+    <t>RNF-08</t>
+  </si>
+  <si>
+    <t>Seguridad (Concurrencia)</t>
+  </si>
+  <si>
+    <t>El sistema deberá forzar la invalidación inmediata de sesiones activas al detectar una nueva conexión del mismo usuario desde otro cliente, cumpliendo la política de dispositivo único.</t>
+  </si>
+  <si>
+    <t>Tiempo de invalidación y revocación de credenciales activas en Redis menor a 500 ms tras una nueva autenticación concurrente detectada.</t>
+  </si>
+  <si>
+    <t>RNF-09</t>
+  </si>
+  <si>
+    <t>Capacidad de monitoreo</t>
+  </si>
+  <si>
+    <t>El sistema deberá emitir y almacenar trazas de auditoría inmutables para garantizar trazabilidad y no repudio frente a accesos, rechazos y eventos de esteganografía (RSG-07, RSG-15).</t>
+  </si>
+  <si>
+    <t>El 100% de los incidentes de seguridad e intentos anómalos deben ser transmitidos a Syslog remoto/SIEM en menos de 1 s con encadenamiento criptográfico de hashes para verificar su no alteración.</t>
+  </si>
+  <si>
+    <t>RNF-10</t>
+  </si>
+  <si>
+    <t>Mantenibilidad (Shift Left)</t>
+  </si>
+  <si>
+    <t>El código fuente de la aplicación debe cumplir con estándares de codificación segura (ISO/IEC 27034, NIST SP 800-218) auditados de forma continua en el pipeline de integración continua.</t>
+  </si>
+  <si>
+    <t>Cero vulnerabilidades críticas o altas (según OWASP Top 10) reportadas por escáneres SAST y pruebas de dependencias en el repositorio antes del despliegue a producción.</t>
+  </si>
+  <si>
+    <t>RNF-11</t>
+  </si>
+  <si>
+    <t>Usabilidad</t>
+  </si>
+  <si>
+    <t>Las interfaces de usuario y paneles administrativos deben proveer retroalimentación visual clara e inequívoca sobre el estado de la conexión, aforo y resultado del análisis de adjuntos.</t>
+  </si>
+  <si>
+    <t>Tiempo de inducción operativa para el administrador inferior a 15 minutos y tasa de error en la parametrización de salas inferior al 5% en pruebas de usabilidad guiadas.</t>
+  </si>
+  <si>
+    <t>RNF-12</t>
+  </si>
+  <si>
+    <t>Interoperabilidad</t>
+  </si>
+  <si>
+    <t>El sistema debe implementar estándares abiertos y protocolos estándar para el transporte en tiempo real e intercambio de datos, evitando librerías binarias cerradas.</t>
+  </si>
+  <si>
+    <t>Cumplimiento estricto del estándar W3C WebSockets (RFC 6455), HTTP/2 y payloads de comunicación codificados en formato estándar JSON (RFC 8259).</t>
+  </si>
+  <si>
+    <t>Umbral</t>
+  </si>
+  <si>
+    <t>Tiempo de entrega de mensaje menor a 200 ms en el percentil 95 (P95) bajo una carga de hasta 100 usuarios concurrentes por sala.</t>
+  </si>
+  <si>
+    <t>Latencia &lt;= 200 ms (P95)</t>
+  </si>
+  <si>
+    <t>MTTD &lt;= 1.5 s (archivos &lt;= 5 MB)</t>
+  </si>
+  <si>
+    <t>Uptime &gt;= 99.5% mensual</t>
+  </si>
+  <si>
+    <t>Capacidad &gt;= 500 conexiones / 50 salas (CPU &lt;= 75%, RAM &lt;= 80%)</t>
+  </si>
+  <si>
+    <t>RTO &lt;= 60 s</t>
+  </si>
+  <si>
+    <t>TLS 1.3 estricto (Calificación 'A')</t>
+  </si>
+  <si>
+    <t>100% contenedores no-root y read-only rootfs</t>
+  </si>
+  <si>
+    <t>Revocación de sesión &lt;= 500 ms</t>
+  </si>
+  <si>
+    <t>Cobertura = 100% eventos, Latencia &lt;= 1 s</t>
+  </si>
+  <si>
+    <t>0 vulnerabilidades críticas/altas</t>
+  </si>
+  <si>
+    <t>Tiempo &lt;= 15 min / Error &lt;= 5%</t>
+  </si>
+  <si>
+    <t>100% cumplimiento RFC 6455, HTTP/2, RFC 8259</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -231,18 +437,97 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -258,14 +543,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{02002C2F-326A-524B-8251-65C7FB2D741A}" name="Tabla1" displayName="Tabla1" ref="A1:E15" totalsRowShown="0">
-  <autoFilter ref="A1:E15" xr:uid="{02002C2F-326A-524B-8251-65C7FB2D741A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{02002C2F-326A-524B-8251-65C7FB2D741A}" name="Tabla1" displayName="Tabla1" ref="A1:E15" totalsRowShown="0" headerRowDxfId="11">
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{5378A4C4-8F57-CB4D-B54D-0BAA407D321B}" name="Código"/>
-    <tableColumn id="2" xr3:uid="{108C7AE4-79FE-AD4E-9736-C034505FB9AE}" name="Requisito funcional"/>
-    <tableColumn id="3" xr3:uid="{519C8EEA-1BCF-C34B-B1B6-560683174AB7}" name="Descripción" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{CB7AAC04-F313-F545-A9A3-42737FDFF59D}" name="Actor"/>
-    <tableColumn id="5" xr3:uid="{80444791-1C20-9445-B07E-6287FB55F0FC}" name="Prioridad"/>
+    <tableColumn id="1" xr3:uid="{5378A4C4-8F57-CB4D-B54D-0BAA407D321B}" name="Código" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{108C7AE4-79FE-AD4E-9736-C034505FB9AE}" name="Requisito funcional" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{519C8EEA-1BCF-C34B-B1B6-560683174AB7}" name="Descripción" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{CB7AAC04-F313-F545-A9A3-42737FDFF59D}" name="Actor" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{80444791-1C20-9445-B07E-6287FB55F0FC}" name="Prioridad" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{19013AE0-5517-CE4E-8921-66D026070E37}" name="Tabla2" displayName="Tabla2" ref="A1:E13" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:E13" xr:uid="{19013AE0-5517-CE4E-8921-66D026070E37}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{B15C1987-E253-C547-8E16-061A382017E0}" name="Código" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{702BF794-1CDB-444F-8F29-A3F97944F5FC}" name="Atributo" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{22CD9E22-00A1-7449-9A20-F604249B7AE9}" name="Requisito no funcional" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{9F1E2F0E-93BF-4C4D-ACA6-96A5D55BC4FD}" name="Criterio de aceptación" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{5D92A5A5-3149-5040-B6FD-EB92F9204BD1}" name="Umbral" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -594,261 +892,261 @@
     <col min="2" max="2" width="43" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="80.33203125" customWidth="1"/>
     <col min="4" max="4" width="25.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="A12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="A13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="A14" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="4" t="s">
         <v>48</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="A15" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="4" t="s">
         <v>51</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="4" t="s">
         <v>16</v>
       </c>
     </row>
@@ -862,9 +1160,241 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66248F6D-B2B9-AB4C-8C44-0B4A56B85761}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10.1640625" customWidth="1"/>
+    <col min="2" max="2" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.6640625" customWidth="1"/>
+    <col min="4" max="4" width="63.1640625" customWidth="1"/>
+    <col min="5" max="5" width="56.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>